<commit_message>
Add Phase-1 routes slide (1.c) with all 10 routes; update sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XLC7pA91a4QFnpJfEJZnxa
</commit_message>
<xml_diff>
--- a/Hydrogen_Vehicle_Study_Sources.xlsx
+++ b/Hydrogen_Vehicle_Study_Sources.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$3:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$3:$G$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -824,7 +824,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>1.b / 1.c India H2 Pilots</t>
+          <t>1.b / 1.d India H2 Pilots</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>1.b / 1.c India H2 Pilots</t>
+          <t>1.b / 1.d India H2 Pilots</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -923,8 +923,183 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>1.c Phase-1 Routes</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Tata Motors: 16 H2 trucks (Prima H.55S, H.28; H2-ICE &amp; FCEV) on Mumbai, Pune, Delhi-NCR, Surat, Vadodara, Jamshedpur, Kalinganagar routes</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Autocar Pro</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Tata Motors begins hydrogen truck trials in India</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>https://autocarpro.in/news/tata-motors-begins-hydrogen-truck-trials-in-india-125235</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>1.c Phase-1 Routes</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Tata pilot with Indian Oil; NGHM allocation to Tata, RIL, NTPC, Ashok Leyland, HPCL, BPCL, IOCL</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Business Standard</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>India's vehicles industry quietly begins shift to hydrogen-powered vehicles</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.business-standard.com/industry/auto/indian-cv-majors-drive-hydrogen-transition-with-h2-vehicles-125061600725_1.html</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>16 Jun 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>1.c Phase-1 Routes</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Kerala (ANERT): 4 trucks, HRS at Muttathara &amp; Udyogamandal (260 kg/day), Ashok Leyland, BPCL, Greenstat, KSRTC; Rs 34.84 cr</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Construction World</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Kerala secures Rs 34.84 crore for green hydrogen transport pilot</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>https://www.constructionworld.in/energy-infrastructure/power-and-renewable-energy/kerala-secures-rs-34.84-crore-for-green-hydrogen-transport-pilot/67306</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>1.c Phase-1 Routes</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Odisha: NTPC 3 hydrogen buses with CRUT &amp; GRIDCO; 42 seats, 600 km range; H2 plant at CRUT depot</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>The Week (PTI)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Odisha signs agreement to operate hydrogen-powered buses</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.theweek.in/wire-updates/national/2024/12/24/ces2-od-hydrogen-bus.html</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>24 Dec 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>1.c Phase-1 Routes</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>10 routes list; IOCL HRS at Faridabad R&amp;D and Vadodara; scheme guidelines</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Rajya Sabha (eParliament)</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Unstarred question AU5278 – reply</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>https://eparlib.sansad.in/bitstream/123456789/3010203/1/AU5278_ccyEJc.pdf</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:G14"/>
+  <autoFilter ref="A3:G19"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
@@ -937,6 +1112,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete Hydrogen Vehicle Study deck: add slides 2–25 mirroring EV deck; fix 1.c route mapping per Lok Sabha Q1648; update sources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XLC7pA91a4QFnpJfEJZnxa
</commit_message>
<xml_diff>
--- a/Hydrogen_Vehicle_Study_Sources.xlsx
+++ b/Hydrogen_Vehicle_Study_Sources.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$3:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sources'!$A$3:$G$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1098,8 +1098,883 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>1.c, 1.d, 2, 4 – Pilots &amp; stations</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Official route-to-consortium mapping, vehicles and ₹ sanctioned for all 12 pilots; 70 vehicles (27 buses, 43 trucks), 16 HRS, ₹410.77 cr</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Lok Sabha (MNRE reply)</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Unstarred Q1648 – hydrogen vehicle pilots</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>https://sansad.in/getFile/lsapps/loksabhaquestions/annex/188/AU1648_XD1qA0.pdf</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>29 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>2 – Policy (NGHM)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>SIGHT 3,000 MW/yr to 15 cos; 8.62 lakh TPA awarded, ~8,000 TPA running; pilot, hub, R&amp;D outlays; hubs &amp; HVICs; skilling</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>PIB</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>National Green Hydrogen Mission progress</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>https://www.pib.gov.in/PressReleseDetailm.aspx?PRID=2329321&amp;reg=48&amp;lang=2</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>2 – Policy (NGHM)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Component outlays: SIGHT ₹17,490 cr, pilots ₹1,466 cr, R&amp;D ₹400 cr, other ₹388 cr</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>narendramodi.in (Cabinet release)</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Cabinet approves National Green Hydrogen Mission</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.narendramodi.in/cabinet-approves-national-green-hydrogen-mission-566866</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>4 Jan 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>ICE vs BEV vs FCEV; H₂ types; H₂-ICE</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>FC tank-to-wheel 40–50%; H₂-ICE conversion, injection 10–20 / up to 350 bar, NOx, cost; HRS cost 5–6× CNG</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>EVreporter</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Hydrogen ICE vehicles and their relevance in commercial mobility</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>https://evreporter.com/hydrogen-ice-vehicles-and-their-relevance-in-commercial-mobility/</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>3.a, 8, 12, 20 – Mirai Gen-2</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>128 kW stack, 330 cells, 5.6 kg H₂, 3 tanks, 134 kW motor, 84-cell battery 31.5 kW/10 s, −30 °C start, FDC</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Toyota UK Magazine</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>New Mirai hydrogen fuel cell vehicle – under the skin</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>https://mag.toyota.co.uk/new-mirai-hydrogen-fuel-cell-electric-vehicle/</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>3.a – Generations</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Toyota 2nd-gen FC system: 114→128 kW, 33→24 L, 41→24 kg, 5.4 kW/L, 58% less Pt per output, no humidifier</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>JSME</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>The Second-Generation Toyota Fuel Cell System (award)</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>https://www.jsme.or.jp/english/about/awards/2021-2/award2021-nt2/</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>3.a – Generations</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Nexo Gen-1 vs Gen-2: 95→110 kW, 6.33→6.69 kg, 666→700+ km, battery 1.56→2.64 kWh</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Paultan</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>2025 Hyundai Nexo debuts</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>https://paultan.org/2025/04/03/2025-hyundai-nexo-debuts/</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>3 Apr 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>3.a / Types – Plug-in FCEV</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>CR-V e:FCEV: 17.7 kWh battery, 29-mile EV range, 4.3 kg H₂, 270-mile total</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Green Car Reports</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>2025 Honda CR-V e:FCEV – 29-mile EV range</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>https://www.greencarreports.com/news/1142418_2025-honda-cr-v-fcev-29-mile-ev-range-hydrogen</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>3.a, 14 – History &amp; consumption</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>FCV history (Electrovan 1966, FCX 2002, Clarity 2008, ix35 2013, Mirai 2014, Nexo 2018); MPGe; XCIENT fill time</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Wikipedia</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Fuel cell vehicle</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Fuel_cell_vehicle</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>accessed Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>3.b – Fuel cell types</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Electrolyte, temperature, stack size, efficiency, applications, challenges for PEMFC/AFC/PAFC/MCFC/SOFC</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>US DOE HFTO</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Comparison of Fuel Cell Technologies fact sheet</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>https://www.energy.gov/eere/fuelcells/articles/comparison-fuel-cell-technologies-fact-sheet</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>accessed Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>3.c, 14, 22 – Refuelling</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>350/700 bar, 3–5 min fill, SAE J2601, 85 °C tank limit, ISO 19880-5 hoses, car–station data link</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>Hyfindr</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Complete refuelling line – components</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hyfindr.com/en/hydrogen-knowledge/complete-refueling-line</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>accessed Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>3.c, 12, 17 – Indian H₂ buses</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Tata–IOCL buses: 70 kW FC, 30 kg at 350 bar, 300+ km, ~1 kg/10 km; IOCL Faridabad &amp; Vadodara stations; Leh 80 kg/day</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>The Week</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Why India is betting big on hydrogen buses</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>https://www.theweek.in/theweek/business/2026/05/09/why-india-is-betting-big-on-hydrogen-buses.html</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>9 May 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>15 – Stack manufacturing</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>PEM stack process steps (GDL, catalyst coating, MEA, plates, seals, stacking, conditioning) and challenges</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>US DOE (MYPP)</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Hydrogen &amp; Fuel Cells Multi-Year Program Plan – Manufacturing R&amp;D</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>https://webarchive.library.unt.edu/web/20121007121342/http://www1.eere.energy.gov/hydrogenandfuelcells/mypp/pdfs/manufacturing.pdf</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>3.d – Electrolyser capacity</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>~58 GW/yr factory capacity end-2025, &lt;5 GW output, ~9% utilisation, China 60%/Europe 20%/US 10%, system costs</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Argus Media (IEA GHR 2026)</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Green H2 electrolyser sector enters consolidation – IEA</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.argusmedia.com/en/news-and-insights/latest-market-news/2841836-green-h2-electrolyser-sector-enters-consolidation-iea</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>3.d – Electrolyser capacity</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Installed electrolysis &gt;4 GW (doubled 2025), China ~¾ of new; demand &gt;100 Mt; low-emissions ~1 Mt</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Global Hydrogen Review 2026 – Executive summary</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.iea.org/reports/global-hydrogen-review-2026/executive-summary</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>3.d – SIGHT Tranche I</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Electrolyser manufacturing winners and MW/yr (1,500 MW total)</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Renewable Watch</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>SECI declares winners of its 1.5 GW electrolyser manufacturing auction</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>https://renewablewatch.in/2024/01/16/seci-declares-winners-of-its-1-5-gw-electrolyser-manufacturing-auction/</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>16 Jan 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>4 – Refuelling infra</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>NTPC Leh: 5 FC buses, 80 kg/day station, 1.7 MW solar, 11,562 ft</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>Renewable Watch</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>NTPC deploys five hydrogen fuel cell buses in Leh</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>https://renewablewatch.in/2025/06/20/ntpc-deploys-five-hydrogen-fuel-cell-buses-in-leh/</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>20 Jun 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>4 – Refuelling infra</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>IOCL setting up HRS at Faridabad, Vadodara, Pune, Balasore</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Indian Infrastructure</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Developments in the LNG and green hydrogen segments</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>https://indianinfrastructure.com/2025/08/04/exploring-alternatives-developments-in-the-lng-and-green-hydrogen-segments/</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>4 Aug 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Financing &amp; subsidies</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>GST on fuel cell vehicles cut 12% → 5%</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Electrive</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>India makes fuel cell vehicles cheaper as part of tax reform</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.electrive.com/2025/09/22/india-makes-fuel-cell-vehicles-cheaper-as-part-of-tax-reform</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>22 Sep 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Financing &amp; subsidies</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>7-year permit exemption for hydrogen, electric, ethanol, methanol CVs (AIS-140)</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Autocar Pro</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Electric, ethanol, hydrogen CVs get 7-year permit exemption</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>https://www.autocarpro.in/news/electric-ethanol-hydrogen-cvs-get-7-year-permit-exemption-133500</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>8 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Financing &amp; subsidies</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Korea Nexo subsidy ₩22.5m national + ₩10–12m local; price ₩69.5m; peak 10,527 (2022)</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Hydrogen Insight</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Only two hydrogen cars sold in South Korea despite 50% subsidies</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.hydrogeninsight.com/transport/only-two-hydrogen-cars-sold-in-south-korea-last-month-despite-subsidies-offering-50-discounts/2-1-1602437</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Financing &amp; subsidies</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>China FCV city pilots: rewards to cities, 50,000 FCVs by 2025 goal</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>ICCT</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Ten cities, thousand fuel cell vehicles – China's hydrogen roadmap</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>https://theicct.org/ten-cities-thousand-fuel-cell-vehicles-china-is-sketching-a-roadmap-for-hydrogen-vehicles/</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>accessed Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Critical minerals</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Platinum mine output by country 2025e (South Africa ~71%, Russia ~12%); palladium (Russia ~44%)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>USGS</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Mineral Commodity Summaries 2026 – Platinum-group metals</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>https://pubs.usgs.gov/periodicals/mcs2026/mcs2026-platinum-group.pdf</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Critical minerals</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>South Africa produces ~80% of world iridium</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Mining Weekly (SFA Oxford)</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>South Africa must strengthen key iridium status</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.miningweekly.com/article/south-africa-must-strengthen-key-iridium-status-sfa-oxford-2022-04-29</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>29 Apr 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Thermal &amp; water</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>FCEV stack ≤80 °C, ΔT 40 °C vs ICE 80 °C, 25 kW vs 20 kW heat to coolant, ~2–2.5× cooling (illustrative)</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>FutureBridge</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Navigating thermal challenges in fuel cell EVs</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.futurebridge.com/industry/perspectives-mobility/navigating-thermal-challenges-in-fuel-cell-evs-with-new-innovations/</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>accessed Oct 2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:G19"/>
+  <autoFilter ref="A3:G44"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId2"/>
@@ -1117,6 +1992,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId41"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>